<commit_message>
feat: formato de precios, fondo blanco en imágenes, bundle ID iOS y mejoras UI
- Precios con separador de miles ($255.000) en todas las pantallas via format_utils.dart
- Imágenes de producto con fondo blanco (BoxFit.contain + container blanco)
- Alineación de imagen ajustada en miniaturas (Alignment -0.4)
- Bundle ID actualizado a com.okventa.app en proyecto iOS
- Correcciones en email_publisher: identificación por email remitente, URLs imágenes
- Plantilla Excel actualizada con columnas ESTADO, SKU, CODIGO UNIVERSAL

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/resources/OkVenta_Plantilla_Publicaciones.xlsx
+++ b/backend/resources/OkVenta_Plantilla_Publicaciones.xlsx
@@ -8,9 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="Publicaciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="_Listas" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Instrucciones" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="Electr_nica">'_Listas'!$C$1:$C$7</definedName>
+    <definedName name="Automotriz">'_Listas'!$D$1:$D$4</definedName>
+    <definedName name="Hogar">'_Listas'!$E$1:$E$3</definedName>
+    <definedName name="Ocio">'_Listas'!$F$1:$F$3</definedName>
+    <definedName name="Mascotas">'_Listas'!$G$1:$G$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -34,6 +41,13 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00555555"/>
       <sz val="10"/>
@@ -43,12 +57,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="002E7D32"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -80,17 +88,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FDECEA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007B1F1F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -155,16 +163,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -178,7 +186,7 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -258,6 +266,110 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>OkVenta</author>
+  </authors>
+  <commentList>
+    <comment ref="A5" authorId="0" shapeId="0">
+      <text>
+        <t>TÍTULO DEL PRODUCTO ✏️
+USA UN TÍTULO LLAMATIVO Y BREVE PARA VENDER TU PRODUCTO.
+Ejemplo: Lente Canon 50mm f/1.8 — Como nuevo
+Máximo 80 caracteres.</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>PRECIO (CLP) 💰
+Solo números enteros en pesos chilenos.
+Sin puntos, comas ni símbolos $.
+Ejemplo: 85000</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>ESTADO DEL PRODUCTO 🏷️
+Selecciona de la lista ▼
+• NUEVO → Producto sin uso, en caja o con etiqueta
+• USADO → Producto en uso, puede tener desgaste</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>CATEGORÍA 📦
+Selecciona de la lista desplegable ▼
+Opciones: Electrónica, Automotriz, Hogar, Ocio, Mascotas.</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>SUBCATEGORÍA 🗂️
+Primero selecciona CATEGORIA.
+Luego elige la subcategoría correspondiente ▼</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>IMAGEN PRINCIPAL 🔗 (obligatoria)
+1. Ve a https://postimages.org/es/
+2. Sube tu foto
+3. Copia el link directo
+4. Pégalo aquí
+Ejemplo: https://i.postimg.cc/xxx/foto.jpg</t>
+      </text>
+    </comment>
+    <comment ref="G5" authorId="0" shapeId="0">
+      <text>
+        <t>DESCRIPCIÓN 📝
+DESCRIBE TU PRODUCTO DETALLADAMENTE
+(ORIGEN, MODELO, MARCA, ESTADO, ACCESORIOS, ETC...)
+Si se omite se usará el título.
+Máximo 300 caracteres.</t>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0" shapeId="0">
+      <text>
+        <t>SEGUNDA IMAGEN 🔗 (opcional)
+1. Sube la foto en postimages.org
+2. Copia el link directo
+3. Pégalo aquí</t>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0" shapeId="0">
+      <text>
+        <t>TERCERA IMAGEN 🔗 (opcional)
+1. Sube la foto en postimages.org
+2. Copia el link directo
+3. Pégalo aquí</t>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0" shapeId="0">
+      <text>
+        <t>SKU (opcional)
+Código interno de tu inventario.
+Ejemplo: CAM-001</t>
+      </text>
+    </comment>
+    <comment ref="K5" authorId="0" shapeId="0">
+      <text>
+        <t>CÓDIGO UNIVERSAL (opcional)
+Código de barras o código universal del producto.
+Ejemplo: 4902505394188</t>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="0" shapeId="0">
+      <text>
+        <t>NOTAS INTERNAS (no se publican)
+Apuntes para tu referencia.
+Ejemplo: Revisar precio / Producto de bodega B</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -552,17 +664,17 @@
   <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -573,135 +685,80 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Completa una fila por producto. Las columnas marcadas con * son obligatorias. Adjunta las imágenes al correo con el mismo nombre indicado en las columnas Imagen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="6" customHeight="1"/>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>titulo *</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>precio *</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>descripcion</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>categoria</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>subcategoria</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>user_id *</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>imagen</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>imagen2</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>imagen3</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>lat</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>lng</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Cámara Sony Alpha A7</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>250000</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Cámara mirrorless en excelente estado, incluye cargador</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Electrónica</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Fotografía</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>42</t>
+          <t>📷  Obtén el link de tus imágenes aquí  →  https://postimages.org/es/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Sube tus fotos en postimages.org, copia el link directo y pégalo en las columnas de imagen. Los campos con * son obligatorios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1"/>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TITULO</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>PRECIO</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>ESTADO</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>SUBCATEGORIA</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>IMAGEN_URL</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>camara_sony.jpg</t>
+          <t>DESCRIPCION</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>camara_sony_2.jpg</t>
+          <t>IMAGEN_URL2</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>camara_sony_3.jpg</t>
+          <t>IMAGEN_URL3</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>-33.4569</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>-70.6483</t>
+          <t>CODIGO UNIVERSAL</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Color: negro / sin garantía</t>
+          <t>NOTAS</t>
         </is>
       </c>
     </row>
@@ -1126,11 +1183,39 @@
       <c r="L35" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A3:L3"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
   </mergeCells>
+  <dataValidations count="7">
+    <dataValidation sqref="C6:C35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Estado inválido" error="Selecciona NUEVO o USADO de la lista ▼" promptTitle="Estado del producto" prompt="Selecciona el estado ▼&#10;• NUEVO: sin uso&#10;• USADO: en uso" type="list">
+      <formula1>"NUEVO,USADO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6:D35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Categoría inválida" error="Selecciona de la lista ▼" promptTitle="Categoría" prompt="Selecciona la categoría del producto ▼" type="list">
+      <formula1>_Listas!$A$1:$A$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="E6:E35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Subcategoría inválida" error="Selecciona primero CATEGORIA, luego elige aquí." promptTitle="Subcategoría" prompt="Primero elige CATEGORIA, luego aquí ▼" type="list">
+      <formula1>INDIRECT(SUBSTITUTE(D6," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6:B35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Precio inválido" error="Solo números enteros positivos en CLP. Sin puntos ni símbolos." promptTitle="Precio (CLP)" prompt="Entero positivo. Ejemplo: 85000" type="whole" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="F6:F35" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="🔗 Link de imagen" prompt="Sube tu foto en postimages.org/es/&#10;Copia el link directo y pégalo aquí." type="textLength" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6:H35" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="🔗 Link de imagen" prompt="Sube tu foto en postimages.org/es/&#10;Copia el link directo y pégalo aquí." type="textLength" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="I6:I35" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="🔗 Link de imagen" prompt="Sube tu foto en postimages.org/es/&#10;Copia el link directo y pégalo aquí." type="textLength" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1140,16 +1225,174 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Electrónica</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Fotografía</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Cámaras para auto</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Deportes</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Cámaras para mascotas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Automotriz</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>USADO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Dashcam</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Vigilancia</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Accesorios</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hogar</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Domótica</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Naturaleza</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ocio</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Computación</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mascotas</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Telefonía</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Drones</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Accesorios</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>OkVenta — Guía de uso de la plantilla</t>
+          <t>OkVenta — Guía de uso de la planilla</t>
         </is>
       </c>
     </row>
@@ -1159,176 +1402,236 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>CAMPOS OBLIGATORIOS (*)</t>
+          <t>CÓMO FUNCIONA</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>titulo *    →  Nombre del producto (ej: Lente Canon 50mm f/1.8)</t>
+          <t>1. Sube tus imágenes en postimages.org/es/ y copia el link directo de cada una.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>precio *    →  Solo números, sin puntos ni símbolos (ej: 85000)</t>
+          <t>2. Pega cada link en las columnas IMAGEN_URL, IMAGEN_URL2, IMAGEN_URL3.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>user_id *   →  Tu ID de usuario en OkVenta (consulta al administrador)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="8" customHeight="1">
-      <c r="A7" s="9" t="inlineStr"/>
+          <t>3. Completa las demás columnas del producto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>4. Envía esta planilla por correo a fpinto@galmar.cl</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>5. En menos de 5 minutos tus productos aparecen publicados en la app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Tu cuenta se identifica por el correo desde el que envías la planilla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="8" customHeight="1">
+      <c r="A10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>CAMPOS OBLIGATORIOS (*)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>TITULO      →  Usa un título llamativo y breve para vender tu producto. Máx 80 caracteres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>PRECIO      →  Solo números enteros en CLP. Ejemplo: 85000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>ESTADO      →  Selecciona NUEVO o USADO de la lista ▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>CATEGORIA   →  Selecciona de la lista ▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>SUBCATEGORIA→  Selecciona según la categoría elegida ▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>IMAGEN_URL  →  Link directo de la imagen principal (postimages.org)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="8" customHeight="1">
+      <c r="A18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>CAMPOS OPCIONALES</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>descripcion →  Detalle del producto. Si se omite, se usará el título.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>categoria   →  Ej: Electrónica / Automotriz / Hogar / Ocio / Mascotas</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>subcategoria→  Ej: Fotografía / Iluminación / Accesorios</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>imagen      →  Nombre del archivo de imagen adjunto al correo (ej: foto.jpg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>imagen2/3   →  Segunda y tercera imagen (misma lógica)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>lat / lng   →  Coordenadas GPS opcionales para mostrar en el mapa</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>notas       →  Campo libre, no se publica. Solo referencia interna.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="8" customHeight="1">
-      <c r="A16" s="9" t="inlineStr"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>CÓMO ENVIAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>1. Rellena las filas en la hoja 'Publicaciones' (una fila = un producto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>2. Si tienes fotos, adjúntalas al correo con el mismo nombre que pusiste en 'imagen'.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>3. Envía el correo a fpinto@galmar.cl (o la cuenta configurada).</t>
+          <t>DESCRIPCION     →  Describe tu producto detalladamente (origen, modelo, marca, etc.)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>4. En menos de 5 minutos los productos aparecen publicados en la app.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="8" customHeight="1">
-      <c r="A22" s="11" t="inlineStr"/>
+          <t>IMAGEN_URL2/3   →  Segunda y tercera imagen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>SKU             →  Código interno de tu inventario.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>CATEGORÍAS DISPONIBLES</t>
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>CODIGO UNIVERSAL→  Código de barras o código universal del producto.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Electrónica   → Fotografía, Video, Audio, Computación, Telefonía, Drones, Accesorios</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>Automotriz    → Cámaras para auto, Dashcam, GPS, Seguridad</t>
-        </is>
-      </c>
+          <t>NOTAS           →  Apuntes internos, no se publican.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="8" customHeight="1">
+      <c r="A25" s="9" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>Hogar         → Seguridad, Vigilancia, Domótica</t>
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>CÓMO OBTENER EL LINK DE UNA IMAGEN</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>Ocio          → Deportes, Viajes, Naturaleza</t>
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>1. Ve a https://postimages.org/es/</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>Mascotas      → Cámaras para mascotas, Accesorios</t>
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>2. Haz clic en 'Elegir imágenes' y sube tu foto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>3. Copia el 'Link directo' (termina en .jpg o .png).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>4. Pega ese link en la celda IMAGEN_URL de esta planilla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="8" customHeight="1">
+      <c r="A31" s="11" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>CATEGORÍAS DISPONIBLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Electrónica  → Fotografía, Video, Audio, Computación, Telefonía, Drones, Accesorios</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Automotriz   → Cámaras para auto, Dashcam, GPS, Seguridad</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Hogar        → Seguridad, Vigilancia, Domótica</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>Ocio         → Deportes, Viajes, Naturaleza</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>Mascotas     → Cámaras para mascotas, Accesorios</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="37">
     <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A37:C37"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A3:C3"/>
@@ -1336,21 +1639,29 @@
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A33:C33"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A32:C32"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A35:C35"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A34:C34"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A6:C6"/>

</xml_diff>